<commit_message>
@mars order added in PCBway Cart from eSpark Account .
</commit_message>
<xml_diff>
--- a/Design-Files/Design-v2.1/Deliverables/BOM/Client-BOM-Design-v2.1.xlsx
+++ b/Design-Files/Design-v2.1/Deliverables/BOM/Client-BOM-Design-v2.1.xlsx
@@ -1,15 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\enlilishaya-windmillcircuit\Design-Files\Design-v2.1\Deliverables\BOM\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7620"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7620"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -27,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="249">
   <si>
     <t>#</t>
   </si>
@@ -756,19 +761,31 @@
   </si>
   <si>
     <t>Zetiling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B00224 </t>
+  </si>
+  <si>
+    <t>Sanyo Stepper Motor w/ 17.5mm 20 Tooth Gear - 12 V - 7.5 deg / step - 42mm D</t>
+  </si>
+  <si>
+    <t>Sanyo</t>
+  </si>
+  <si>
+    <t>B00224</t>
+  </si>
+  <si>
+    <t>Battery</t>
+  </si>
+  <si>
+    <t>Battery 2200 mAh</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="27">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -831,147 +848,10 @@
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -990,194 +870,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="16">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -1268,253 +962,14 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1557,74 +1012,34 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="0003A4CB"/>
-      <color rgb="002CD0B2"/>
+      <color rgb="FF03A4CB"/>
+      <color rgb="FF2CD0B2"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1882,28 +1297,29 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K50"/>
+  <dimension ref="A1:K52"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="3.14285714285714" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.7142857142857" style="1" customWidth="1"/>
+    <col min="2" max="2" width="3.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="36" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26.5714285714286" customWidth="1"/>
-    <col min="7" max="7" width="33.4285714285714" customWidth="1"/>
-    <col min="8" max="8" width="21.4285714285714" customWidth="1"/>
-    <col min="9" max="9" width="8.14285714285714" customWidth="1"/>
-    <col min="10" max="10" width="9.28571428571429" customWidth="1"/>
-    <col min="11" max="11" width="11.2857142857143" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" customWidth="1"/>
+    <col min="9" max="9" width="8.140625" customWidth="1"/>
+    <col min="10" max="10" width="9.28515625" customWidth="1"/>
+    <col min="11" max="11" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" spans="1:11">
+    <row r="1" spans="1:11">
       <c r="A1" s="2"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1912,11 +1328,11 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-    </row>
-    <row r="2" ht="15.75" spans="1:11">
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+    </row>
+    <row r="2" spans="1:11">
       <c r="A2" s="2"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -1949,10 +1365,10 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" ht="24.75" spans="1:11">
+    <row r="3" spans="1:11" ht="24">
       <c r="A3" s="2"/>
       <c r="B3" s="7">
-        <f>ROW(B3)-ROW($B$2)</f>
+        <f t="shared" ref="B3:B49" si="0">ROW(B3)-ROW($B$2)</f>
         <v>1</v>
       </c>
       <c r="C3" s="8" t="s">
@@ -1981,10 +1397,10 @@
       </c>
       <c r="K3" s="9"/>
     </row>
-    <row r="4" ht="36.75" spans="1:11">
+    <row r="4" spans="1:11" ht="36">
       <c r="A4" s="2"/>
       <c r="B4" s="7">
-        <f>ROW(B4)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="C4" s="11" t="s">
@@ -2013,10 +1429,10 @@
       </c>
       <c r="K4" s="12"/>
     </row>
-    <row r="5" ht="15.75" spans="1:11">
+    <row r="5" spans="1:11">
       <c r="A5" s="2"/>
       <c r="B5" s="7">
-        <f>ROW(B5)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="C5" s="8" t="s">
@@ -2048,7 +1464,7 @@
     <row r="6" spans="1:11">
       <c r="A6" s="2"/>
       <c r="B6" s="7">
-        <f>ROW(B6)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C6" s="8" t="s">
@@ -2080,7 +1496,7 @@
     <row r="7" spans="1:11">
       <c r="A7" s="2"/>
       <c r="B7" s="7">
-        <f>ROW(B7)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C7" s="8" t="s">
@@ -2112,7 +1528,7 @@
     <row r="8" spans="1:11">
       <c r="A8" s="2"/>
       <c r="B8" s="7">
-        <f>ROW(B8)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C8" s="8" t="s">
@@ -2144,7 +1560,7 @@
     <row r="9" spans="1:11">
       <c r="A9" s="2"/>
       <c r="B9" s="7">
-        <f>ROW(B9)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C9" s="8" t="s">
@@ -2176,7 +1592,7 @@
     <row r="10" spans="1:11">
       <c r="A10" s="2"/>
       <c r="B10" s="7">
-        <f>ROW(B10)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C10" s="8" t="s">
@@ -2208,7 +1624,7 @@
     <row r="11" spans="1:11">
       <c r="A11" s="2"/>
       <c r="B11" s="7">
-        <f>ROW(B11)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C11" s="8" t="s">
@@ -2237,10 +1653,10 @@
       </c>
       <c r="K11" s="9"/>
     </row>
-    <row r="12" ht="24.75" spans="1:11">
+    <row r="12" spans="1:11" ht="24">
       <c r="A12" s="2"/>
       <c r="B12" s="7">
-        <f>ROW(B12)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C12" s="11" t="s">
@@ -2272,7 +1688,7 @@
     <row r="13" spans="1:11">
       <c r="A13" s="2"/>
       <c r="B13" s="7">
-        <f>ROW(B13)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C13" s="8" t="s">
@@ -2301,10 +1717,10 @@
       </c>
       <c r="K13" s="9"/>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" ht="24">
       <c r="A14" s="2"/>
       <c r="B14" s="7">
-        <f>ROW(B14)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C14" s="11" t="s">
@@ -2331,14 +1747,14 @@
       <c r="J14" s="14">
         <v>2</v>
       </c>
-      <c r="K14" s="17" t="s">
+      <c r="K14" s="16" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="2"/>
       <c r="B15" s="7">
-        <f>ROW(B15)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C15" s="8" t="s">
@@ -2370,7 +1786,7 @@
     <row r="16" spans="1:11">
       <c r="A16" s="2"/>
       <c r="B16" s="7">
-        <f>ROW(B16)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C16" s="11" t="s">
@@ -2399,10 +1815,10 @@
       </c>
       <c r="K16" s="12"/>
     </row>
-    <row r="17" ht="24.75" spans="1:11">
+    <row r="17" spans="1:11" ht="24">
       <c r="A17" s="2"/>
       <c r="B17" s="7">
-        <f>ROW(B17)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="C17" s="8" t="s">
@@ -2431,10 +1847,10 @@
       </c>
       <c r="K17" s="9"/>
     </row>
-    <row r="18" ht="24.75" spans="1:11">
+    <row r="18" spans="1:11" ht="24">
       <c r="A18" s="2"/>
       <c r="B18" s="7">
-        <f>ROW(B18)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="C18" s="11" t="s">
@@ -2463,10 +1879,10 @@
       </c>
       <c r="K18" s="12"/>
     </row>
-    <row r="19" ht="36.75" spans="1:11">
+    <row r="19" spans="1:11" ht="36">
       <c r="A19" s="2"/>
       <c r="B19" s="7">
-        <f>ROW(B19)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="C19" s="8" t="s">
@@ -2495,10 +1911,10 @@
       </c>
       <c r="K19" s="9"/>
     </row>
-    <row r="20" ht="48.75" spans="1:11">
+    <row r="20" spans="1:11" ht="48">
       <c r="A20" s="2"/>
       <c r="B20" s="7">
-        <f>ROW(B20)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C20" s="11" t="s">
@@ -2527,10 +1943,10 @@
       </c>
       <c r="K20" s="12"/>
     </row>
-    <row r="21" ht="15.75" spans="1:11">
+    <row r="21" spans="1:11">
       <c r="A21" s="2"/>
       <c r="B21" s="7">
-        <f>ROW(B21)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="C21" s="8" t="s">
@@ -2559,10 +1975,10 @@
       </c>
       <c r="K21" s="9"/>
     </row>
-    <row r="22" ht="24.75" spans="1:11">
+    <row r="22" spans="1:11" ht="36">
       <c r="A22" s="2"/>
       <c r="B22" s="7">
-        <f>ROW(B22)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="C22" s="11" t="s">
@@ -2594,7 +2010,7 @@
     <row r="23" spans="1:11">
       <c r="A23" s="2"/>
       <c r="B23" s="7">
-        <f>ROW(B23)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="C23" s="8" t="s">
@@ -2621,10 +2037,10 @@
       </c>
       <c r="K23" s="9"/>
     </row>
-    <row r="24" ht="24.75" spans="1:11">
+    <row r="24" spans="1:11" ht="24">
       <c r="A24" s="2"/>
       <c r="B24" s="7">
-        <f>ROW(B24)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="C24" s="11" t="s">
@@ -2653,10 +2069,10 @@
       </c>
       <c r="K24" s="12"/>
     </row>
-    <row r="25" ht="15.75" spans="1:11">
+    <row r="25" spans="1:11" ht="24">
       <c r="A25" s="2"/>
       <c r="B25" s="7">
-        <f>ROW(B25)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="C25" s="8" t="s">
@@ -2685,10 +2101,10 @@
       </c>
       <c r="K25" s="9"/>
     </row>
-    <row r="26" ht="15.75" spans="1:11">
+    <row r="26" spans="1:11" ht="24">
       <c r="A26" s="2"/>
       <c r="B26" s="7">
-        <f>ROW(B26)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C26" s="11" t="s">
@@ -2717,10 +2133,10 @@
       </c>
       <c r="K26" s="12"/>
     </row>
-    <row r="27" spans="1:11">
+    <row r="27" spans="1:11" ht="24">
       <c r="A27" s="2"/>
       <c r="B27" s="7">
-        <f>ROW(B27)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="C27" s="8" t="s">
@@ -2749,10 +2165,10 @@
       </c>
       <c r="K27" s="9"/>
     </row>
-    <row r="28" ht="24.75" spans="1:11">
+    <row r="28" spans="1:11" ht="24">
       <c r="A28" s="2"/>
       <c r="B28" s="7">
-        <f>ROW(B28)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="C28" s="11" t="s">
@@ -2781,10 +2197,10 @@
       </c>
       <c r="K28" s="12"/>
     </row>
-    <row r="29" ht="24.75" spans="1:11">
+    <row r="29" spans="1:11" ht="24">
       <c r="A29" s="2"/>
       <c r="B29" s="7">
-        <f>ROW(B29)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="C29" s="8" t="s">
@@ -2813,10 +2229,10 @@
       </c>
       <c r="K29" s="9"/>
     </row>
-    <row r="30" ht="24.75" spans="1:11">
+    <row r="30" spans="1:11" ht="24">
       <c r="A30" s="2"/>
       <c r="B30" s="7">
-        <f>ROW(B30)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="C30" s="11" t="s">
@@ -2848,7 +2264,7 @@
     <row r="31" spans="1:11">
       <c r="A31" s="2"/>
       <c r="B31" s="7">
-        <f>ROW(B31)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>29</v>
       </c>
       <c r="C31" s="8" t="s">
@@ -2880,7 +2296,7 @@
     <row r="32" spans="1:11">
       <c r="A32" s="2"/>
       <c r="B32" s="7">
-        <f>ROW(B32)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C32" s="8" t="s">
@@ -2912,7 +2328,7 @@
     <row r="33" spans="1:11">
       <c r="A33" s="2"/>
       <c r="B33" s="7">
-        <f>ROW(B33)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>31</v>
       </c>
       <c r="C33" s="8" t="s">
@@ -2944,7 +2360,7 @@
     <row r="34" spans="1:11">
       <c r="A34" s="2"/>
       <c r="B34" s="7">
-        <f>ROW(B34)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C34" s="8" t="s">
@@ -2976,7 +2392,7 @@
     <row r="35" spans="1:11">
       <c r="A35" s="2"/>
       <c r="B35" s="7">
-        <f>ROW(B35)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="C35" s="8" t="s">
@@ -3008,7 +2424,7 @@
     <row r="36" spans="1:11">
       <c r="A36" s="2"/>
       <c r="B36" s="7">
-        <f>ROW(B36)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>34</v>
       </c>
       <c r="C36" s="8" t="s">
@@ -3040,7 +2456,7 @@
     <row r="37" spans="1:11">
       <c r="A37" s="2"/>
       <c r="B37" s="7">
-        <f>ROW(B37)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>35</v>
       </c>
       <c r="C37" s="8" t="s">
@@ -3072,7 +2488,7 @@
     <row r="38" spans="1:11">
       <c r="A38" s="2"/>
       <c r="B38" s="7">
-        <f>ROW(B38)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>36</v>
       </c>
       <c r="C38" s="8" t="s">
@@ -3104,7 +2520,7 @@
     <row r="39" spans="1:11">
       <c r="A39" s="2"/>
       <c r="B39" s="7">
-        <f>ROW(B39)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>37</v>
       </c>
       <c r="C39" s="8" t="s">
@@ -3133,10 +2549,10 @@
       </c>
       <c r="K39" s="9"/>
     </row>
-    <row r="40" spans="1:11">
+    <row r="40" spans="1:11" ht="24">
       <c r="A40" s="2"/>
       <c r="B40" s="7">
-        <f>ROW(B40)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>38</v>
       </c>
       <c r="C40" s="8" t="s">
@@ -3163,14 +2579,14 @@
       <c r="J40" s="14">
         <v>1</v>
       </c>
-      <c r="K40" s="17" t="s">
+      <c r="K40" s="16" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="41" spans="1:11">
       <c r="A41" s="2"/>
       <c r="B41" s="7">
-        <f>ROW(B41)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>39</v>
       </c>
       <c r="C41" s="8" t="s">
@@ -3202,7 +2618,7 @@
     <row r="42" spans="1:11">
       <c r="A42" s="2"/>
       <c r="B42" s="7">
-        <f>ROW(B42)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>40</v>
       </c>
       <c r="C42" s="8" t="s">
@@ -3234,7 +2650,7 @@
     <row r="43" spans="1:11">
       <c r="A43" s="2"/>
       <c r="B43" s="7">
-        <f>ROW(B43)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>41</v>
       </c>
       <c r="C43" s="8" t="s">
@@ -3266,7 +2682,7 @@
     <row r="44" spans="1:11">
       <c r="A44" s="2"/>
       <c r="B44" s="7">
-        <f>ROW(B44)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>42</v>
       </c>
       <c r="C44" s="11" t="s">
@@ -3295,10 +2711,10 @@
       </c>
       <c r="K44" s="12"/>
     </row>
-    <row r="45" ht="24.75" spans="1:11">
+    <row r="45" spans="1:11" ht="24">
       <c r="A45" s="2"/>
       <c r="B45" s="7">
-        <f>ROW(B45)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>43</v>
       </c>
       <c r="C45" s="8" t="s">
@@ -3327,10 +2743,10 @@
       </c>
       <c r="K45" s="9"/>
     </row>
-    <row r="46" ht="24.75" spans="1:11">
+    <row r="46" spans="1:11" ht="36">
       <c r="A46" s="2"/>
       <c r="B46" s="7">
-        <f>ROW(B46)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>44</v>
       </c>
       <c r="C46" s="11" t="s">
@@ -3362,7 +2778,7 @@
     <row r="47" spans="1:11">
       <c r="A47" s="2"/>
       <c r="B47" s="7">
-        <f>ROW(B47)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>45</v>
       </c>
       <c r="C47" s="8" t="s">
@@ -3394,7 +2810,7 @@
     <row r="48" spans="1:11">
       <c r="A48" s="2"/>
       <c r="B48" s="7">
-        <f>ROW(B48)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>46</v>
       </c>
       <c r="C48" s="11" t="s">
@@ -3423,10 +2839,10 @@
       </c>
       <c r="K48" s="12"/>
     </row>
-    <row r="49" ht="24.75" spans="1:11">
+    <row r="49" spans="1:11" ht="24">
       <c r="A49" s="2"/>
       <c r="B49" s="7">
-        <f>ROW(B49)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>47</v>
       </c>
       <c r="C49" s="8" t="s">
@@ -3455,7 +2871,7 @@
       </c>
       <c r="K49" s="9"/>
     </row>
-    <row r="50" ht="15.75" spans="2:11">
+    <row r="50" spans="1:11" ht="15.75" thickBot="1">
       <c r="B50" s="7">
         <v>48</v>
       </c>
@@ -3484,13 +2900,80 @@
         <v>10</v>
       </c>
       <c r="K50" s="9"/>
+    </row>
+    <row r="51" spans="1:11" ht="36.75" thickBot="1">
+      <c r="B51" s="7">
+        <v>48</v>
+      </c>
+      <c r="C51" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="D51" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E51" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="F51" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G51" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="H51" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="I51" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J51" s="9">
+        <v>1</v>
+      </c>
+      <c r="K51" s="18" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="15.75" thickBot="1">
+      <c r="B52" s="7">
+        <v>48</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E52" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="F52" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G52" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H52" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="I52" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J52" s="9">
+        <v>1</v>
+      </c>
+      <c r="K52" s="18" t="s">
+        <v>247</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="I1:K1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="K51" r:id="rId1"/>
+    <hyperlink ref="K52" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Client BOM Update and order placed to PCBway cart.
</commit_message>
<xml_diff>
--- a/Design-Files/Design-v2.1/Deliverables/BOM/Client-BOM-Design-v2.1.xlsx
+++ b/Design-Files/Design-v2.1/Deliverables/BOM/Client-BOM-Design-v2.1.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="248">
   <si>
     <t>#</t>
   </si>
@@ -775,10 +775,7 @@
     <t>B00224</t>
   </si>
   <si>
-    <t>Battery</t>
-  </si>
-  <si>
-    <t>Battery 2200 mAh</t>
+    <t>B07TKL2JRM</t>
   </si>
 </sst>
 </file>
@@ -797,14 +794,14 @@
       <sz val="10"/>
       <color indexed="13"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -812,27 +809,27 @@
       <sz val="10"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -840,7 +837,7 @@
       <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -848,6 +845,7 @@
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -1015,11 +1013,11 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1304,7 +1302,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K52"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="1" customWidth="1"/>
@@ -1328,9 +1326,9 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="2"/>
@@ -2871,7 +2869,7 @@
       </c>
       <c r="K49" s="9"/>
     </row>
-    <row r="50" spans="1:11" ht="15.75" thickBot="1">
+    <row r="50" spans="1:11" ht="30.75" thickBot="1">
       <c r="B50" s="7">
         <v>48</v>
       </c>
@@ -2899,7 +2897,9 @@
       <c r="J50" s="9">
         <v>10</v>
       </c>
-      <c r="K50" s="9"/>
+      <c r="K50" s="17" t="s">
+        <v>247</v>
+      </c>
     </row>
     <row r="51" spans="1:11" ht="36.75" thickBot="1">
       <c r="B51" s="7">
@@ -2929,40 +2929,8 @@
       <c r="J51" s="9">
         <v>1</v>
       </c>
-      <c r="K51" s="18" t="s">
+      <c r="K51" s="17" t="s">
         <v>246</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" ht="15.75" thickBot="1">
-      <c r="B52" s="7">
-        <v>48</v>
-      </c>
-      <c r="C52" s="8" t="s">
-        <v>239</v>
-      </c>
-      <c r="D52" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E52" s="10" t="s">
-        <v>248</v>
-      </c>
-      <c r="F52" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="G52" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H52" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="I52" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="J52" s="9">
-        <v>1</v>
-      </c>
-      <c r="K52" s="18" t="s">
-        <v>247</v>
       </c>
     </row>
   </sheetData>
@@ -2971,7 +2939,7 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="K51" r:id="rId1"/>
-    <hyperlink ref="K52" r:id="rId2"/>
+    <hyperlink ref="K50" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>